<commit_message>
Restore source-backed N. meningitidis limits and metric display consistency
</commit_message>
<xml_diff>
--- a/public/static/summary/species_counts.xlsx
+++ b/public/static/summary/species_counts.xlsx
@@ -7634,14 +7634,28 @@
           <t>qualibact-v1.1</t>
         </is>
       </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>warn</t>
+        </is>
+      </c>
       <c r="D208" t="n">
-        <v>32386</v>
+        <v>32116</v>
       </c>
       <c r="E208" t="n">
-        <v>32259</v>
+        <v>31977</v>
       </c>
       <c r="F208" t="n">
-        <v>127</v>
+        <v>139</v>
+      </c>
+      <c r="G208" t="n">
+        <v>30660</v>
+      </c>
+      <c r="H208" t="n">
+        <v>3240</v>
+      </c>
+      <c r="I208" t="n">
+        <v>1916</v>
       </c>
     </row>
     <row r="209">

</xml_diff>